<commit_message>
Mueve Retiro #122 a Julio y agrega cache busting (?v=) en CSS/JS
Renueva la versión automáticamente en cada ejecución de actualizar.py,
para que los visitantes siempre reciban la última versión del calendario.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/16. CALENDARIO - EL VIVE/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC0D2FF6-4F2D-4E5C-97B2-40D590DFAD9D}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C6D4C5B-FC59-4B0F-B56D-F1F555EDBF19}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -921,7 +921,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
Apostolados mensuales sin día exacto: muestra "por definir" en vez de casilla vacía
Los apostolados de jul-dic quedan sin día en el Excel (fecha y lugar por
definir). El render muestra un icono 📅 con "por definir" y ya no se atenúan
como eventos pasados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/16. CALENDARIO - EL VIVE/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C6D4C5B-FC59-4B0F-B56D-F1F555EDBF19}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51F99779-5377-40A7-BA65-331F778C15E1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="79">
   <si>
     <t>Mes</t>
   </si>
@@ -258,6 +258,9 @@
   </si>
   <si>
     <t>Retiro #122 de Monterrey</t>
+  </si>
+  <si>
+    <t>Lugar y fecha exacta por definir</t>
   </si>
 </sst>
 </file>
@@ -859,12 +862,8 @@
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="2">
-        <v>18</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
         <v>15</v>
       </c>
@@ -872,7 +871,9 @@
         <v>22</v>
       </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="3"/>
+      <c r="G10" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1011,12 +1012,8 @@
       <c r="A17" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="2">
-        <v>22</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
       <c r="D17" s="2" t="s">
         <v>15</v>
       </c>
@@ -1024,7 +1021,9 @@
         <v>22</v>
       </c>
       <c r="F17" s="2"/>
-      <c r="G17" s="3"/>
+      <c r="G17" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1183,12 +1182,8 @@
       <c r="A25" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B25" s="2">
-        <v>19</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
       <c r="D25" s="2" t="s">
         <v>15</v>
       </c>
@@ -1196,7 +1191,9 @@
         <v>22</v>
       </c>
       <c r="F25" s="2"/>
-      <c r="G25" s="3"/>
+      <c r="G25" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="H25" s="2"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1309,12 +1306,8 @@
       <c r="A31" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="2">
-        <v>17</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
       <c r="D31" s="2" t="s">
         <v>15</v>
       </c>
@@ -1322,7 +1315,9 @@
         <v>22</v>
       </c>
       <c r="F31" s="2"/>
-      <c r="G31" s="3"/>
+      <c r="G31" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1473,12 +1468,8 @@
       <c r="A39" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="2">
-        <v>7</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
       <c r="D39" s="2" t="s">
         <v>15</v>
       </c>
@@ -1486,7 +1477,9 @@
         <v>22</v>
       </c>
       <c r="F39" s="2"/>
-      <c r="G39" s="3"/>
+      <c r="G39" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="H39" s="2"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -1597,12 +1590,8 @@
       <c r="A45" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="2">
-        <v>5</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
       <c r="D45" s="2" t="s">
         <v>15</v>
       </c>
@@ -1610,7 +1599,9 @@
         <v>22</v>
       </c>
       <c r="F45" s="2"/>
-      <c r="G45" s="3"/>
+      <c r="G45" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="H45" s="2"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Apostolado mensual de Junio: ahora es el martes 30 de junio
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/16. CALENDARIO - EL VIVE/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51F99779-5377-40A7-BA65-331F778C15E1}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BC660EF-8540-4F0C-92EE-58E62BFD2253}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="80">
   <si>
     <t>Mes</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t>Lugar y fecha exacta por definir</t>
+  </si>
+  <si>
+    <t>Lugar y hora por definir</t>
   </si>
 </sst>
 </file>
@@ -759,19 +762,21 @@
         <v>8</v>
       </c>
       <c r="B5" s="2">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>79</v>
+      </c>
       <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Agregar Retiro de Compromiso INI#1 (27-29 nov) desde Excel
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/16. CALENDARIO - EL VIVE/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BC660EF-8540-4F0C-92EE-58E62BFD2253}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E241FDE-E939-4134-92DA-1354A66B1A27}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="83">
   <si>
     <t>Mes</t>
   </si>
@@ -167,9 +167,6 @@
     <t>(O apostolado con KIDS, por definir.)</t>
   </si>
   <si>
-    <t>Limpieza de rancho</t>
-  </si>
-  <si>
     <t>Diciembre</t>
   </si>
   <si>
@@ -264,6 +261,18 @@
   </si>
   <si>
     <t>Lugar y hora por definir</t>
+  </si>
+  <si>
+    <t>27-29</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>Retiro de Compromiso</t>
+  </si>
+  <si>
+    <t>Retiro de compromiso INI#1 HMO</t>
   </si>
 </sst>
 </file>
@@ -775,7 +784,7 @@
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2"/>
     </row>
@@ -877,7 +886,7 @@
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H10" s="2"/>
     </row>
@@ -886,20 +895,20 @@
         <v>16</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>29</v>
@@ -930,20 +939,20 @@
         <v>16</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>29</v>
@@ -1027,7 +1036,7 @@
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H17" s="2"/>
     </row>
@@ -1100,20 +1109,20 @@
         <v>35</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>29</v>
@@ -1197,7 +1206,7 @@
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H25" s="2"/>
     </row>
@@ -1321,7 +1330,7 @@
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H31" s="2"/>
     </row>
@@ -1483,7 +1492,7 @@
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H39" s="2"/>
     </row>
@@ -1555,25 +1564,29 @@
       <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="2">
-        <v>28</v>
+      <c r="B43" s="2" t="s">
+        <v>79</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="F43" s="2"/>
-      <c r="G43" s="3"/>
-      <c r="H43" s="2"/>
+      <c r="G43" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B44" s="2">
         <v>2</v>
@@ -1593,7 +1606,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1605,13 +1618,13 @@
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H45" s="2"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B46" s="2">
         <v>8</v>
@@ -1623,7 +1636,7 @@
         <v>32</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="3"/>
@@ -1631,19 +1644,19 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="2">
         <v>11</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F47" s="2"/>
       <c r="G47" s="3"/>
@@ -1651,7 +1664,7 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B48" s="2">
         <v>12</v>
@@ -1663,7 +1676,7 @@
         <v>26</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="3"/>
@@ -1671,7 +1684,7 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" s="2">
         <v>14</v>
@@ -1683,17 +1696,17 @@
         <v>26</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H49" s="2"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B50" s="2">
         <v>16</v>
@@ -1713,19 +1726,19 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B51" s="2">
         <v>17</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="3"/>
@@ -1758,7 +1771,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1766,57 +1779,57 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
@@ -1824,7 +1837,7 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mover Retiro de Compromiso INI#1 a diciembre 4-6 desde Excel
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/16. CALENDARIO - EL VIVE/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E241FDE-E939-4134-92DA-1354A66B1A27}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="11_D4A95994B4412ECF0EA6A1973DF75AD389D62E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82BB3DBD-1644-42AB-BF5D-6A2A73A7A0CB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="82">
   <si>
     <t>Mes</t>
   </si>
@@ -261,9 +261,6 @@
   </si>
   <si>
     <t>Lugar y hora por definir</t>
-  </si>
-  <si>
-    <t>27-29</t>
   </si>
   <si>
     <t>Si</t>
@@ -1562,47 +1559,47 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>79</v>
+        <v>47</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="F43" s="2"/>
-      <c r="G43" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>80</v>
-      </c>
+      <c r="G43" s="3"/>
+      <c r="H43" s="2"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="2">
-        <v>2</v>
+      <c r="B44" s="2" t="s">
+        <v>69</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="F44" s="2"/>
-      <c r="G44" s="3"/>
-      <c r="H44" s="2"/>
+      <c r="G44" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">

</xml_diff>

<commit_message>
Apostolado mensual movido al 1 de julio + aviso de reprogramación
Nueva columna "Reprogramado" (Sí/No) en el Excel; muestra el badge
"Reprogramado · cambio de fecha" en el evento marcado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -482,6 +482,7 @@
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.95" customHeight="1">
@@ -530,6 +531,11 @@
           <t>Ubicación (Google Maps)</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Reprogramado</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -559,6 +565,7 @@
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="3" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -588,6 +595,7 @@
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="3" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -617,19 +625,20 @@
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="3" t="n"/>
-    </row>
-    <row r="5">
+      <c r="J4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -645,13 +654,18 @@
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Lugar y hora por definir</t>
+          <t>Hospital General del Estado (Blvd. Colosio y Quintero Arce)</t>
         </is>
       </c>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/wZGdSHUt6B2ged2w8</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -683,6 +697,7 @@
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="3" t="n"/>
+      <c r="J6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -720,6 +735,7 @@
       </c>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="3" t="n"/>
+      <c r="J7" s="2" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -749,6 +765,7 @@
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="3" t="n"/>
+      <c r="J8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -778,6 +795,7 @@
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="3" t="n"/>
+      <c r="J9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -805,6 +823,7 @@
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="3" t="n"/>
+      <c r="J10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -844,6 +863,7 @@
         </is>
       </c>
       <c r="I11" s="3" t="n"/>
+      <c r="J11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -873,6 +893,7 @@
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="3" t="n"/>
+      <c r="J12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -912,6 +933,7 @@
         </is>
       </c>
       <c r="I13" s="3" t="n"/>
+      <c r="J13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -951,6 +973,7 @@
         </is>
       </c>
       <c r="I14" s="3" t="n"/>
+      <c r="J14" s="2" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -980,6 +1003,7 @@
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="3" t="n"/>
+      <c r="J15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1009,6 +1033,7 @@
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="3" t="n"/>
+      <c r="J16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1036,6 +1061,7 @@
       </c>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="3" t="n"/>
+      <c r="J17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1065,6 +1091,7 @@
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="3" t="n"/>
+      <c r="J18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1102,6 +1129,7 @@
       </c>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="3" t="n"/>
+      <c r="J19" s="2" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1131,6 +1159,7 @@
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="3" t="n"/>
+      <c r="J20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1170,6 +1199,7 @@
         </is>
       </c>
       <c r="I21" s="3" t="n"/>
+      <c r="J21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1207,6 +1237,7 @@
       </c>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="3" t="n"/>
+      <c r="J22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1236,6 +1267,7 @@
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="3" t="n"/>
+      <c r="J23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1265,6 +1297,7 @@
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="3" t="n"/>
+      <c r="J24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1292,6 +1325,7 @@
       </c>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="3" t="n"/>
+      <c r="J25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1321,6 +1355,7 @@
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="3" t="n"/>
+      <c r="J26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1358,6 +1393,7 @@
       </c>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="3" t="n"/>
+      <c r="J27" s="2" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -1387,6 +1423,7 @@
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="3" t="n"/>
+      <c r="J28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1416,6 +1453,7 @@
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="3" t="n"/>
+      <c r="J29" s="2" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -1449,6 +1487,7 @@
       </c>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="3" t="n"/>
+      <c r="J30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1476,6 +1515,7 @@
       </c>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="3" t="n"/>
+      <c r="J31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1505,6 +1545,7 @@
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="3" t="n"/>
+      <c r="J32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1534,6 +1575,7 @@
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="3" t="n"/>
+      <c r="J33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1571,6 +1613,7 @@
       </c>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="3" t="n"/>
+      <c r="J34" s="2" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -1600,6 +1643,7 @@
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="3" t="n"/>
+      <c r="J35" s="2" t="n"/>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -1629,6 +1673,7 @@
       <c r="G36" s="3" t="n"/>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="3" t="n"/>
+      <c r="J36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1658,6 +1703,7 @@
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="3" t="n"/>
+      <c r="J37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1687,6 +1733,7 @@
       <c r="G38" s="3" t="n"/>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="3" t="n"/>
+      <c r="J38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1714,6 +1761,7 @@
       </c>
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="3" t="n"/>
+      <c r="J39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1751,6 +1799,7 @@
       </c>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="3" t="n"/>
+      <c r="J40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1780,6 +1829,7 @@
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="2" t="n"/>
       <c r="I41" s="3" t="n"/>
+      <c r="J41" s="2" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -1809,6 +1859,7 @@
       <c r="G42" s="3" t="n"/>
       <c r="H42" s="2" t="n"/>
       <c r="I42" s="3" t="n"/>
+      <c r="J42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1838,6 +1889,7 @@
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="3" t="n"/>
+      <c r="J43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1877,6 +1929,7 @@
         </is>
       </c>
       <c r="I44" s="3" t="n"/>
+      <c r="J44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1904,6 +1957,7 @@
       </c>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="3" t="n"/>
+      <c r="J45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1933,6 +1987,7 @@
       <c r="G46" s="3" t="n"/>
       <c r="H46" s="2" t="n"/>
       <c r="I46" s="3" t="n"/>
+      <c r="J46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1962,6 +2017,7 @@
       <c r="G47" s="3" t="n"/>
       <c r="H47" s="2" t="n"/>
       <c r="I47" s="3" t="n"/>
+      <c r="J47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1991,6 +2047,7 @@
       <c r="G48" s="3" t="n"/>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="3" t="n"/>
+      <c r="J48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2024,6 +2081,7 @@
       </c>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="3" t="n"/>
+      <c r="J49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2053,6 +2111,7 @@
       <c r="G50" s="3" t="n"/>
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="3" t="n"/>
+      <c r="J50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2082,10 +2141,11 @@
       <c r="G51" s="3" t="n"/>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="3" t="n"/>
+      <c r="J51" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H52"/>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="A2:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
     </dataValidation>
@@ -2093,6 +2153,9 @@
       <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Misas mensuales vuelven a domingo (no sábado)
Misas mensuales movidas de sábado a domingo (Ago 30, Sep 6, Sep 27,
Oct 25, Nov 15). Regenerado desde el Excel (app.js, eventos.json, .ics).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -1100,11 +1100,11 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H19" s="2" t="n"/>
@@ -1208,11 +1208,11 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H22" s="2" t="n"/>
@@ -1364,11 +1364,11 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H27" s="2" t="n"/>
@@ -1584,11 +1584,11 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H34" s="2" t="n"/>
@@ -1770,11 +1770,11 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">

</xml_diff>